<commit_message>
Calificaciones P00-P02: .class validos (se piden junto con .java) e instrucciones sin nombres
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P02-corte-03sep.xlsx
+++ b/calificaciones/P00-P02-corte-03sep.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +54,11 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -135,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -164,14 +169,17 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -568,14 +576,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Rúbrica:  10 = correcta vía PR   ·   9 = vía PR con detalle de forma (ver Notas)   ·   PC = pendiente de corrección (busca la hoja con tu cuenta)   ·   NP = no presentada</t>
+          <t>Rúbrica:  10 = correcta vía PR   ·   9 = vía PR con detalle de forma (ver Notas)   ·   PC = pendiente de corrección (busca la pestaña con tu cuenta)   ·   NP = no presentada</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Nota: los PRs correctos ya fueron mergeados a main el 03-sep. Si tu estado es PC, tu hoja (pestaña con tu número de cuenta) trae las instrucciones exactas.</t>
+          <t>Los PRs correctos ya fueron mergeados a main el 03-sep. Recuerda: se entregan los .java Y los .class.</t>
         </is>
       </c>
     </row>
@@ -667,7 +675,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>3 ramas pusheadas SIN PR y archivos fuera de la carpeta propia (incluye .class).  →  ver pestaña «323297291»</t>
+          <t>3 ramas pusheadas SIN PR y archivos fuera de la carpeta propia.  →  ver pestaña «323297291»</t>
         </is>
       </c>
     </row>
@@ -749,7 +757,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Completa y correcta. Acción menor: cerrar el PR duplicado (#35); las entregas van en #2/#3/#9.  →  ver pestaña «319012543»</t>
+          <t>Completa y correcta. Acción menor: cerrar el PR duplicado (#35); las entregas ya se mergearon en #2/#3/#9.  →  ver pestaña «319012543»</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1015,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Trabajo completo y muy bien hecho en 3 ramas, pero SIN abrir ningún PR; p02 incluye .class.  →  ver pestaña «322179684»</t>
+          <t>Trabajo completo y muy bien hecho en 3 ramas (los .java y .class están bien), pero SIN abrir ningún PR.  →  ver pestaña «322179684»</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -1450,159 +1458,80 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>P00, P01 y P02 completas en 3 ramas — el contenido está MUY bien (tu p02 con constructores y métodos es de las más completas del grupo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>P00, P01 y P02 completas en 3 ramas — el contenido está MUY bien (tu p02 es de las más completas del grupo, y tus .java y .class están correctos: ambos se entregan).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>• No abriste ningún pull request: el push existe, pero la entrega formal ES el PR.</t>
+          <t>Qué hay que corregir</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>• Tu p02 incluye archivos .class compilados (no se versionan).</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>• No abriste ningún pull request: el push existe, pero la entrega formal ES el PR. Es lo ÚNICO que falta.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Cómo corregirlo, paso a paso</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>1 · Quita los .class de tu p02</t>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Abre los 3 PRs (en el navegador — no necesitas terminal)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>cd mpoo-2027-1</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>entra a tu clon</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>git checkout p02-hernandez-aviña</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>cámbiate a tu rama de p02</t>
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Por cada una de tus tres ramas (la de p00, la de p01 y la de p02): github.com/OscarRuiz21/mpoo-2027-1 → Pull requests → New pull request → base: main ← compare: TU-RAMA → Create pull request. Son 3 PRs, uno por práctica.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>git pull origin p02-hernandez-aviña</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>trae tu última versión</t>
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Al terminar</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>git rm entregas/hernandez_karen/p02/metodos/PruebaPunto.class entregas/hernandez_karen/p02/metodos/Punto.class</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>elimina los compilados del control de versiones</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>git commit -m "P02: fuera archivos compilados"</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>guarda el arreglo</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>git push origin p02-hernandez-aviña</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>súbelo</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>2 · Abre los 3 PRs (en el navegador)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>Por cada rama — p00-hernandez-aviña, p01-hernandez-aviña, p02-hernandez-aviña — Pull requests → New → base: main ← compare: (la rama) → Create pull request. Son 3 PRs, uno por práctica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Al terminar</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>Tu trabajo ya está hecho; solo falta formalizarlo. Con los PRs abiertos, las tres van directo a 10.</t>
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Tu trabajo ya está hecho y muy bien; solo falta formalizarlo. Con los PRs abiertos, las tres van directo a 10.</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -1639,176 +1568,183 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>P00, P01 y P02 en tu rama (P01-Ajas-Andre), bien estructuradas en tu carpeta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>P00, P01 y P02 en una sola rama, bien estructuradas en tu carpeta.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
+          <t>Qué hay que corregir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
           <t>• No abriste el pull request: el push existe, pero la entrega formal ES el PR.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>• Tu p02 trae el ejemplo de la demo de clase; la práctica 2 pide los ejemplos Punto.java y PruebaPunto.java.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>• Tu p02 trae el ejemplo de la demo de clase; la práctica 2 pide los ejemplos Punto.java y PruebaPunto.java (con sus .class).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Cómo corregirlo, paso a paso</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>1 · Corrige el contenido de tu p02</t>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
+          <t>1 · Corrige el contenido de tu p02</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
           <t>cd mpoo-2027-1</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>entra a tu clon del repositorio</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>git checkout P01-Ajas-Andre</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>cámbiate a tu rama (la que ya subiste)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>git pull origin P01-Ajas-Andre</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>git pull origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>asegúrate de tener tu última versión</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>git rm entregas/ajas_andre/p02/Circulo.java</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>git rm entregas/tu_apellido_nombre/p02/Circulo.java</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>elimina el archivo que no corresponde a la P02</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>Copia tus archivos Punto.java y PruebaPunto.java (los de la práctica) a entregas/ajas_andre/p02/</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>git add entregas/ajas_andre/p02/</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Copia tus archivos Punto.java y PruebaPunto.java (con sus .class) a entregas/tu_apellido_nombre/p02/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/p02/</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>prepara los archivos nuevos para el commit</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>git commit -m "P02: ejemplos Punto de la practica"</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>guarda el cambio con un mensaje claro</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>git push origin P01-Ajas-Andre</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>git push origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>sube la corrección a GitHub</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>2 · Abre el pull request (en el navegador)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>github.com/OscarRuiz21/mpoo-2027-1 → Pull requests → New pull request → base: main ← compare: P01-Ajas-Andre → Create pull request. Contesta la plantilla.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Al terminar</t>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>github.com/OscarRuiz21/mpoo-2027-1 → Pull requests → New pull request → base: main ← compare: TU-RAMA → Create pull request. Contesta la plantilla.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Al terminar</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>Con el PR abierto, tus tres prácticas entran a revisión en esa misma entrega.</t>
         </is>
@@ -1847,267 +1783,267 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>P00, P01 y P02 pusheadas en 3 ramas — pero los archivos quedaron sueltos en entregas/ (sin tu carpeta) y subiste los .class compilados. Tampoco abriste PRs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>P00, P01 y P02 pusheadas en 3 ramas — pero los archivos quedaron sueltos en entregas/, sin tu carpeta. Tampoco abriste PRs. (Los .java y .class están bien: ambos se entregan.)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>• Cada quien trabaja SOLO dentro de su carpeta: entregas/apellido_nombre/p00, p01, p02.</t>
+          <t>Qué hay que corregir</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>• Los .class no se versionan: son archivos compilados que se regeneran.</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>• Cada quien trabaja SOLO dentro de su carpeta: entregas/tu_apellido_nombre/p00, p01, p02.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>• Sin PR no hay entrega formal.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Cómo corregirlo, paso a paso</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>1 · Crea una rama nueva y limpia desde main</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>cd mpoo-2027-1</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>entra a tu clon del repositorio</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>git checkout main</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>párate en main</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>trae lo más nuevo antes de empezar</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>git checkout -b p02-bravo</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>git checkout -b p02-tu-apellido</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>crea tu rama de corrección partiendo de main limpio</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>2 · Reconstruye tu estructura de carpetas</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>mkdir -p entregas/bravo_paulo/p00 entregas/bravo_paulo/p01 entregas/bravo_paulo/p02</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>mkdir -p entregas/tu_apellido_nombre/p00 entregas/tu_apellido_nombre/p01 entregas/tu_apellido_nombre/p02</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>crea tus tres carpetas de práctica</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>git checkout p00-Paulo_Bravo -- entregas/Bravo_Paulo.txt</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>recupera tu archivo de la P00 desde tu rama vieja</t>
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA-p00 -- entregas/TuArchivo.txt</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>recupera tu txt de la P00 (el que quedó suelto) desde tu rama vieja</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/Bravo_Paulo.txt entregas/bravo_paulo/p00/bravo_paulo.txt</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/TuArchivo.txt entregas/tu_apellido_nombre/p00/</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>muévelo a su lugar</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>git checkout p01-Paulo_Bravo -- entregas/HolaMundo.java</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>recupera tu HolaMundo (solo el .java, el .class no)</t>
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA-p01 -- entregas/HolaMundo.java entregas/HolaMundo.class</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>recupera tu HolaMundo: el .java y el .class (ambos se entregan)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/HolaMundo.java entregas/bravo_paulo/p01/HolaMundo.java</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>muévelo a tu carpeta p01</t>
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/HolaMundo.java entregas/HolaMundo.class entregas/tu_apellido_nombre/p01/</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>muévelos a tu carpeta p01</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>git checkout p02-Paulo_Bravo -- 'entregas/ejemplo*.java'</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>recupera tus 5 ejemplos (.java solamente)</t>
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA-p02 -- 'entregas/ejemplo*'</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>recupera tus 5 ejemplos: .java y .class</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/ejemplo1.java entregas/ejemplo2.java entregas/ejemplo3.java entregas/ejemplo4.java entregas/ejemplo5.java entregas/bravo_paulo/p02/</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>muévelos a tu carpeta p02</t>
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/ejemplo1.java entregas/ejemplo1.class entregas/ejemplo2.java entregas/ejemplo2.class entregas/ejemplo3.java entregas/ejemplo3.class entregas/ejemplo4.java entregas/ejemplo4.class entregas/ejemplo5.java entregas/ejemplo5.class entregas/tu_apellido_nombre/p02/</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>muévelos (los 10 archivos) a tu carpeta p02</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>3 · Sube y abre el PR</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>git add -A entregas/</t>
         </is>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>registra todos los movimientos</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>git commit -m "P00-P02: reestructura en entregas/bravo_paulo"</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>git commit -m "P00-P02: reestructura en mi carpeta"</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>un commit con el arreglo completo</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>git push origin p02-bravo</t>
-        </is>
-      </c>
-      <c r="B33" s="17" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>git push origin p02-tu-apellido</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>sube tu rama nueva</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>En GitHub: Pull requests → New → base: main ← compare: p02-bravo → Create. Las 3 prácticas entran en este PR.</t>
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>En GitHub: Pull requests → New → base: main ← compare: p02-tu-apellido → Create. Las 3 prácticas entran en este PR.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>Al terminar</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>Tus ramas viejas las borramos después de mergear; no subas nada más a ellas.</t>
         </is>
@@ -2125,7 +2061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -2146,248 +2082,255 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
           <t>P01 (HolaMundo en la RAÍZ del repo) y P02 (carpeta correcta) — pero tus PRs #8 y #33 arrastran archivos del curso: README.md, guias/ y material/. Falta tu P00.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
+          <t>Qué hay que corregir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
           <t>• Tus ramas nacieron de un punto viejo y tocan archivos que no son tuyos: así NO se pueden mergear.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>• Tu HolaMundo debe vivir en entregas/angel_castillo/p01/, no en la raíz.</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>• Tu HolaMundo debe vivir en entregas/tu_apellido_nombre/p01/, no en la raíz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>• Falta la P00 (archivo de prueba con tu nombre).</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Cómo corregirlo, paso a paso</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>1 · Rama nueva desde main limpio, rescatando solo lo tuyo</t>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
+          <t>1 · Rama nueva desde main limpio, rescatando solo lo tuyo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
           <t>cd mpoo-2027-1</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>entra a tu clon</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>git checkout main</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>párate en main</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>trae lo más nuevo</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>git checkout -b p02-castillo</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>git checkout -b p02-tu-apellido</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>rama nueva partiendo de main LIMPIO</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>git checkout p02-Castillo -- entregas/angel_castillo/</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA-DEL-PR-33 -- entregas/tu_apellido_nombre/</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>trae SOLO tu carpeta desde tu rama anterior (nada más)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>git checkout entrega-lab0 -- HolaMundo.java</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA-DEL-PR-8 -- HolaMundo.java</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>rescata tu HolaMundo de la otra rama</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>mkdir -p entregas/angel_castillo/p01</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>mkdir -p entregas/tu_apellido_nombre/p01</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>crea tu carpeta p01</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>git mv HolaMundo.java entregas/angel_castillo/p01/HolaMundo.java</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>git mv HolaMundo.java entregas/tu_apellido_nombre/p01/HolaMundo.java</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>muévelo a TU carpeta, no a la raíz</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>mkdir -p entregas/angel_castillo/p00</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>mkdir -p entregas/tu_apellido_nombre/p00</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>crea tu carpeta p00</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>echo "Apellidos Nombre(s)" &gt; entregas/angel_castillo/p00/nombre.txt</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>echo "Apellidos Nombre(s)" &gt; entregas/tu_apellido_nombre/p00/nombre.txt</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>crea tu archivo de la P00 — escribe TU nombre completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>2 · Sube y reemplaza tus PRs</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
+          <t>2 · Sube y reemplaza tus PRs</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
           <t>git add -A entregas/</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>registra todo</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>git commit -m "P00-P02: entrega completa, rama limpia"</t>
         </is>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>un solo commit limpio</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>git push origin p02-castillo</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>git push origin p02-tu-apellido</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>sube la rama nueva</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>En GitHub abre el PR nuevo (base: main ← compare: p02-castillo) y CIERRA los PRs #8 y #33 (Close pull request), comentando que este los reemplaza.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t>Al terminar</t>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>En GitHub abre el PR nuevo (base: main ← compare: p02-tu-apellido) y CIERRA los PRs #8 y #33 (Close pull request), comentando que este los reemplaza.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Al terminar</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>Con eso tus tres prácticas quedan en un PR limpio que sí se puede revisar y mergear.</t>
         </is>
@@ -2405,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -2426,71 +2369,78 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
           <t>P00, P01 y P02 completas y correctas (calif. 10 las tres) — ya mergeadas a main. Solo queda un duplicado administrativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
+          <t>Qué hay que corregir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
           <t>• Tu PR #35 (la rama con todo junto) duplica a los PRs #2, #3 y #9 que ya se mergearon.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Cómo corregirlo, paso a paso</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Única acción (en el navegador, 1 minuto)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Entra al PR #35 y ciérralo con Close pull request, comentando que las entregas ya se mergearon en #2, #3 y #9.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Al terminar</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Al terminar</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Tus tres prácticas ya están en main con 10. Buen trabajo — estructura y contenido impecables.</t>
         </is>
@@ -2502,6 +2452,422 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF8F00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Corrección · cuenta 322098930</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Revisión: 03-sep-2026, 13:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>P00 (PR #15) y P01 (PR #16). El contenido está bien; el problema es de carpetas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Qué hay que corregir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>• Entre tus dos PRs la P00 existe DOS veces (carpetas P0 y P00): al mergear quedarían duplicadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>• La convención es minúsculas: p00, p01, p02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>• Falta la P02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Cómo corregirlo, paso a paso</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>1 · Normaliza carpetas en tu rama del PR #16</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>cd mpoo-2027-1</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>entra a tu clon</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>cámbiate a la rama de tu PR #16</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>git pull origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>trae tu última versión</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/tu_apellido_nombre/P00 entregas/tu_apellido_nombre/tmp00</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>renombrar solo mayúsculas confunde a macOS/Windows: primero a un nombre temporal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/tu_apellido_nombre/tmp00 entregas/tu_apellido_nombre/p00</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>…y ahora al definitivo en minúsculas</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/tu_apellido_nombre/P1 entregas/tu_apellido_nombre/p01</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>renombra P1 a p01</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>git commit -m "P00-P01: carpetas en minusculas"</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>guarda el arreglo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>git push origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>el PR #16 se actualiza solo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>2 · Cierra el PR duplicado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Tu p00 ya viaja dentro del PR #16: entra al PR #15 y ciérralo (Close pull request).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>3 · Entrega tu P02</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>En la MISMA rama crea entregas/tu_apellido_nombre/p02/ con tus ejemplos Punto (con .java y .class), haz add + commit + push, y el PR #16 llevará las tres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Al terminar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Con eso un solo PR limpio lleva todo tu trabajo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF8F00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Corrección · cuenta 323294506</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Revisión: 03-sep-2026, 13:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>P00 y P02 correctas (ya mergeadas a main, calif. 10). P01 en el PR #31 con carpeta distinta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Qué hay que corregir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>• Tu P01 vive en una carpeta con GUION (apellido-nombre), pero tus otras entregas usan guion bajo (apellido_nombre): al mergear quedarían DOS carpetas tuyas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Cómo corregirlo, paso a paso</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Renombra la carpeta en la rama del PR #31</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>cd mpoo-2027-1</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>entra a tu clon</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>cámbiate a la rama de tu PR #31</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>git pull origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>trae tu última versión</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/tu-apellido-nombre entregas/tu_apellido_nombre</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>renombra TU carpeta: cambia el guion (-) por guion bajo (_)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>git commit -m "P01: carpeta con guion bajo"</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>guarda el arreglo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>git push origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>el PR #31 se actualiza solo, no hay que abrir otro</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Al terminar</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>Con ese rename tu P01 también queda en 10.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FF8F00"/>
@@ -2518,7 +2884,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Corrección · cuenta 322098930</t>
+          <t>Corrección · cuenta 323290577</t>
         </is>
       </c>
     </row>
@@ -2529,597 +2895,202 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>P00 (PR #15) y P01 (PR #16). El contenido está bien; el problema es de carpetas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>P01 (HolaMundo.java) en tu rama. Tu PR #5 se cerró sin mergear y no abriste uno nuevo.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>• Entre tus dos PRs la P00 existe DOS veces (carpetas P0 y P00): al mergear quedarían duplicadas.</t>
+          <t>Qué hay que corregir</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>• La convención es minúsculas: p00, p01, p02.</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>• Sin PR abierto no hay entrega formal: hay que reabrir.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>• Falta la P02.</t>
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>• Faltan P00 y P02.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Cómo corregirlo, paso a paso</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>1 · Normaliza carpetas en tu rama del PR #16</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>cd mpoo-2027-1</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>entra a tu clon</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>git checkout p01-crisostomo</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>cámbiate a la rama de tu PR #16</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>git pull origin p01-crisostomo</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>trae tu última versión</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/crisostomo_israel/P00 entregas/crisostomo_israel/tmp00</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>renombrar solo mayúsculas confunde a macOS/Windows: primero a un nombre temporal</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/crisostomo_israel/tmp00 entregas/crisostomo_israel/p00</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>…y ahora al definitivo en minúsculas</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/crisostomo_israel/P1 entregas/crisostomo_israel/p01</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>renombra P1 a p01</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>git commit -m "P00-P01: carpetas en minusculas"</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>guarda el arreglo</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>git push origin p01-crisostomo</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>el PR #16 se actualiza solo</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>2 · Cierra el PR duplicado</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>Tu p00 ya viaja dentro del PR #16: entra al PR #15 y ciérralo (Close pull request).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>3 · Entrega tu P02</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>En la MISMA rama crea entregas/crisostomo_israel/p02/ con tus ejemplos Punto, haz add + commit + push, y el PR #16 llevará las tres.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>Al terminar</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="13" t="inlineStr">
-        <is>
-          <t>Con eso un solo PR limpio lleva todo tu trabajo.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00FF8F00"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="72" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Corrección · cuenta 323294506</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Revisión: 03-sep-2026, 13:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>P00 y P02 correctas (ya mergeadas a main, calif. 10). P01 en el PR #31 con carpeta distinta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>• Tu P01 vive en una carpeta con GUION (flores-diego), pero tus otras entregas usan guion bajo (flores_diego): al mergear quedarían DOS carpetas tuyas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Cómo corregirlo, paso a paso</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Renombra la carpeta en la rama del PR #31</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>cd mpoo-2027-1</t>
-        </is>
-      </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>entra a tu clon</t>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>git checkout p01-flores</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>cámbiate a la rama de tu PR #31</t>
+          <t>1 · Completa tu P00 en la misma rama</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>git pull origin p01-flores</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>cd mpoo-2027-1</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>entra a tu clon</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>cámbiate a tu rama (la que ya subiste)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>git pull origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>trae tu última versión</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/flores-diego entregas/flores_diego</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>renombra la carpeta: guion bajo, como tus otras entregas</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>git commit -m "P01: carpeta con guion bajo"</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>guarda el arreglo</t>
-        </is>
-      </c>
-    </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>git push origin p01-flores</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>el PR #31 se actualiza solo, no hay que abrir otro</t>
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>mkdir -p entregas/tu_apellido_nombre/p00</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>crea tu carpeta p00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>echo "Apellidos Nombre(s)" &gt; entregas/tu_apellido_nombre/p00/nombre.txt</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>tu archivo de prueba — escribe TU nombre completo</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Al terminar</t>
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/p00</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>prepáralo</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>Con ese rename tu P01 también queda en 10.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00FF8F00"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="72" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Corrección · cuenta 323290577</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Revisión: 03-sep-2026, 13:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>P01 (HolaMundo.java) en tu rama. Tu PR #5 se cerró sin mergear y no abriste uno nuevo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>• Sin PR abierto no hay entrega formal: hay que reabrir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>• Faltan P00 y P02.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Cómo corregirlo, paso a paso</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>1 · Completa tu P00 en la misma rama</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>cd mpoo-2027-1</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>entra a tu clon</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>git checkout Gonzalez_Luis</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>cámbiate a tu rama</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>git pull origin Gonzalez_Luis</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>trae tu última versión</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>mkdir -p entregas/Gonzalez_Luis/p00</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>crea tu carpeta p00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>echo "Apellidos Nombre(s)" &gt; entregas/Gonzalez_Luis/p00/nombre.txt</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>tu archivo de prueba — escribe TU nombre completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>git add entregas/Gonzalez_Luis/p00</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>prepáralo</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>git commit -m "P00: prueba de push"</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>guárdalo</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>git push origin Gonzalez_Luis</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>git push origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>súbelo</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>2 · Abre el PR (en el navegador)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>github.com/OscarRuiz21/mpoo-2027-1 → Pull requests → New → base: main ← compare: Gonzalez_Luis → Create pull request.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>github.com/OscarRuiz21/mpoo-2027-1 → Pull requests → New → base: main ← compare: TU-RAMA → Create pull request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>3 · P02</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
-        <is>
-          <t>En la misma rama crea tu carpeta p02/ con los ejemplos Punto de la práctica, add + commit + push, y el mismo PR la incluirá.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Al terminar</t>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>En la misma rama crea tu carpeta p02/ con los ejemplos Punto (con .java y .class), add + commit + push, y el mismo PR la incluirá.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Al terminar</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>Un solo PR con tus tres prácticas y quedas al corriente.</t>
         </is>
@@ -3137,7 +3108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -3158,183 +3129,190 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Qué entregaste</t>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Privacidad: donde el comando diga TU-RAMA o tu_apellido_nombre, escribe el nombre REAL de tu rama y de tu carpeta (tú los conoces).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
+          <t>Qué entregaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
           <t>P00 y P01 pusheadas en tu rama — sin PR, con la carpeta nombrada con tu usuario y la subcarpeta p1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Qué hay que corregir</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
+          <t>Qué hay que corregir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
           <t>• La carpeta debe llamarse apellido_nombre (primer apellido + primer nombre, minúsculas), no tu usuario de GitHub.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>• La subcarpeta de la práctica 1 es p01, no p1.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>• No abriste el PR.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>• Falta la P02.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Cómo corregirlo, paso a paso</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>(columna A: el comando tal cual en la terminal · columna B: qué está haciendo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>1 · Renombra carpetas en tu rama</t>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>(columna A: el comando en la terminal · columna B: qué está haciendo)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
         <is>
+          <t>1 · Renombra carpetas en tu rama</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
           <t>cd mpoo-2027-1</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>entra a tu clon</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>git checkout p00-AngelUriel654</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>cámbiate a tu rama</t>
-        </is>
-      </c>
-    </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>git pull origin p00-AngelUriel654</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>cámbiate a tu rama (la que ya subiste)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>git pull origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>trae tu última versión</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/AngelUriel654 entregas/gonzalez_ramon</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>la carpeta lleva apellido_nombre</t>
-        </is>
-      </c>
-    </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>git mv entregas/gonzalez_ramon/p1 entregas/gonzalez_ramon/p01</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/TuUsuarioDeGitHub entregas/tu_apellido_nombre</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>la carpeta lleva apellido_nombre, no tu usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>git mv entregas/tu_apellido_nombre/p1 entregas/tu_apellido_nombre/p01</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>las carpetas de práctica van p00, p01, p02</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>git commit -m "P00-P01: carpeta apellido_nombre y p01"</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>guarda el arreglo</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>git push origin p00-AngelUriel654</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>git push origin TU-RAMA</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>súbelo</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>2 · Abre el PR y entrega P02</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>En GitHub: Pull requests → New → base: main ← compare: p00-AngelUriel654 → Create. Después, en la misma rama, agrega tu p02/ con los ejemplos Punto (add + commit + push) y el PR llevará las tres.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Al terminar</t>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>En GitHub: Pull requests → New → base: main ← compare: TU-RAMA → Create. Después, en la misma rama, agrega tu p02/ con los ejemplos Punto (add + commit + push) y el PR llevará las tres.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Al terminar</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>Con el rename y el PR abierto quedas en revisión.</t>
         </is>

</xml_diff>